<commit_message>
feat: Actualizar archivo de instalación de telemetría AiM para Triumph 675 SR
</commit_message>
<xml_diff>
--- a/Plan_Instalacion_Telemetria_AiM_CFMoto675SR.xlsx
+++ b/Plan_Instalacion_Telemetria_AiM_CFMoto675SR.xlsx
@@ -12,8 +12,25 @@
     <sheet name="03_Checklist" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="04_Materiales" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="05_Piezas_3D_Futuro" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="06_BOM_Compras" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="07_STL_Encontrados" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Especificaciones'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'01_Especificaciones'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Protocolo_SOP'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'02_Protocolo_SOP'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Checklist'!$A$1:$D$24</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'03_Checklist'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Materiales'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'04_Materiales'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Piezas_3D_Futuro'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'05_Piezas_3D_Futuro'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_BOM_Compras'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'06_BOM_Compras'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'07_STL_Encontrados'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'07_STL_Encontrados'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,16 +46,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +73,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,242 +477,244 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Sistema / Componente</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ubicacion Tecnica</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Fijacion / Torque</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Herramientas / Materiales</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Calibracion / Notas Criticas</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>QC (Check)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>AiM EVO4 (Modulo Central)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Subchasis / Bandeja trasera</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Velcro 3M Dual Lock + Bridas</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Desengrasante, Nivel de burbuja</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Alinear ejes X/Y/Z con la moto. Nivelacion a 0 deg estricta.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MyChron3 Dash (Display)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Cockpit / Arana mecanizada</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Tornilleria M6 (10 Nm) + Loctite 243</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Llave dinamometrica, llaves Allen</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Comprobar visibilidad en posicion de acople del piloto.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Antena GPS</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Colin / Frontal (Cupula)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Cinta 3M VHB</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Alcohol isopropilico para limpieza</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Sin obstruccion superior (carbono/metal bloquean senal).</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Potenciometro (Suspension)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Horquilla delantera</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Abrazaderas M4 (3-4 Nm)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Pie de rey, llaves Allen 3mm</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Reservar min. 5mm de vastago en compresion maxima.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Sensor Velocidad (Inductivo)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Soporte pinza freno radial</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Tornilleria M6 (10 Nm) + Loctite 243</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Galgas de espesores</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Gap milimetrico de 1.0 - 2.0 mm respecto al disco.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Mazo de Cables / CAN Bus</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Ramal principal chasis</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Cinta de tela (Tesa) / Bridas</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Pasacables, funda termorretractil</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Aislar de fuentes de interferencia electromagnetica.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -687,291 +736,293 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Tarea Especifica</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Especificaciones Tecnicas (El Como)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Verificacion y Control de Calidad (QC)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Tiempo Est.</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Firma</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1. Prep</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Aislamiento electrico</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Desconectar borne negativo de la bateria.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Voltaje 0V confirmado en el sistema.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>1. Prep</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Desmontaje carenados</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Retirar plasticos para acceso al chasis.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Tornilleria en bandejas magneticas numeradas.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2. Core</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Montaje de Datalogger</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Instalar EVO4 con tolerancias de vibracion.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Nivel confirmado a 0 deg en ejes longitudinal/transversal.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2. Core</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Montaje Dash y GPS</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Adherir GPS tras desengrasar; atornillar Dash.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Giro del manillar libre de topes; cables sin tension.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>3. Sens</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Regulacion Potenciometro</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Alinear vastago 100% paralelo a la barra.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Test fisico: Hundir a tope, verificar que no colapsa.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>3. Sens</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Regulacion Velocidad</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Ajustar distancia sensor-tornillo del disco.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Giro manual 360 deg: Lectura positiva en todos los tornillos.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>25 min</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>4. Cabl</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Enrutamiento seguro</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Guiar mazo principal por el interior del chasis.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Cables alejados &gt;5cm de colectores y sin pinzamiento.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>5. Soft</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Setup RaceStudio</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Dar contacto, cargar configuracion de 675 SR.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Pilotos LED de EVO4 encendidos, conexion a PC estable.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>5. Soft</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Calibracion a Cero</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Establecer 0 de suspension extendida.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Telemetria en vivo mostrando valores reales y logicos.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>15 min</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -991,443 +1042,445 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Tarea Especifica</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Accion Detallada y Precauciones</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Fase 1: Preparacion</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Desconectar la bateria</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Retirar el borne negativo para evitar cortocircuitos.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Fase 1: Preparacion</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Desmontaje de carenados</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Retirar tapas laterales, asiento, colin y cupula frontal.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fase 1: Preparacion</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Presentacion en seco</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Colocar provisionalmente los elementos para medir longitud de cables.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Fase 2: Modulo EVO4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Fijacion del EVO4</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Instalar en subchasis asegurando 100% horizontalidad.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Fase 2: Modulo EVO4</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Aislamiento de vibraciones</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Usar velcro industrial o silentblocks para proteger el disco interno.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Fase 2: Modulo EVO4</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Toma de corriente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Conectar a 12V bajo llave y asegurar buena masa.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Fase 3: Cockpit y GPS</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Soporte del Dash</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Fabricar/adaptar pletina de aluminio o carbono.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Fase 3: Cockpit y GPS</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Fijacion de la pantalla</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Guiar cable rizado sin que interfiera con el giro del manillar.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Fase 3: Cockpit y GPS</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Ubicacion de antena GPS</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Pegar con cinta 3M de doble cara en colin o cupula.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Fase 3: Cockpit y GPS</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Verificacion de vision</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Comprobar vision directa al cielo sin obstrucciones.</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Fase 4: Sensores</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Soportes del potenciometro</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Instalar abrazaderas en botella y soporte de pinza.</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Fase 4: Sensores</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Alineacion del potenciometro</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sensor debe trabajar completamente paralelo a la horquilla.</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Fase 4: Sensores</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>PRUEBA CRITICA (Recorrido)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Comprimir horquilla a tope; el sensor NO debe llegar a su limite.</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Fase 4: Sensores</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Soporte sensor de velocidad</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Fabricar pletina en pinza de freno (trasera pref.).</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Fase 4: Sensores</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Ajuste del Gap (Velocidad)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Ajustar distancia a 1.0 - 2.0 mm con galga.</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Fase 5: Enrutado y ECU</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Guiado limpio</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Pasar cables pegados a vigas principales con bridas.</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Fase 5: Enrutado y ECU</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Proteccion termica/mecanica</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Distancia &gt;5cm de colectores y libre de puntos de giro.</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Fase 5: Enrutado y ECU</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Conexion a ECU</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Conectar CAN Bus a OBD o cable inductivo a bobina.</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Fase 6: Config y Pruebas</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Conectar bateria</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Verificar que EVO4 y Dash encienden correctamente.</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Fase 6: Config y Pruebas</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Conexion a PC</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Abrir AiM RaceStudio en el portatil.</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Fase 6: Config y Pruebas</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Configuracion de Moto</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Configurar modelo de moto y protocolo CAN.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Fase 6: Config y Pruebas</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Calibracion a Cero</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Calibrar punto Cero con la moto extendida en caballetes.</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Fase 6: Config y Pruebas</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Prueba de giro</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Girar rueda manualmente y verificar lectura de velocidad.</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1448,331 +1501,333 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Material / Pieza</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Especificacion Tecnica</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Cantidad Est.</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Proposito de Instalacion</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Soportes</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Pletina de Aluminio</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Grado 6061-T6 (2mm)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>1 unidad</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Soportes de Dash y Sensor Velocidad.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Soportes</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Abrazaderas de Horquilla</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Anillos mecanizados a medida</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2 unidades</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Anclaje de potenciometro a suspension.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Tornilleria</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Kit Tornilleria Inox</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Acero Inox A2 (M4, M5, M6)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>1 kit</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Fijacion de herrajes y sensores.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Fijacion</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Velcro Industrial</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>3M Dual Lock</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>20 cm</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Sujecion de EVO4 y Dash.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Fijacion</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Adhesivo Doble Cara</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>3M VHB (Very High Bond)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>1 rollo</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Fijacion de antena GPS.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Proteccion</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cinta de Tela (Tesa)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Estilo OEM (Motorcycle)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>1 rollo</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Proteccion mazo de cables contra roces.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Proteccion</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Tubo Termorretractil</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Con adhesivo interno</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>1 kit</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Sellado estanco de conexiones.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Gestion</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Bridas de Nylon</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Resistentes UV/Calor</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>50 unidades</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Organizacion del cableado por el chasis.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Quimicos</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Fijador de Roscas</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Loctite 243 (Azul)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>1 bote</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Seguridad contra vibraciones del motor.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Quimicos</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Limpiador Superficies</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Alcohol Isopropilico</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>1 bote</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Limpieza previa de zonas de contacto.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Electrico</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Porta-fusible aereo</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Mini-blade (Fusible 5A)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>1 unidad</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Proteccion linea de alimentacion.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1797,268 +1852,870 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Pieza 3D</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Zona de montaje</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Objetivo funcional</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Material recomendado</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Proceso sugerido</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Tolerancia objetivo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Estado CAD</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Archivo STL</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notas de impresion</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Soporte Dash frontal</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Arana frontal</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Reducir vibracion y facilitar lectura</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>PA12</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>SLS</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>+/-0.20 mm</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Insertos metalicos para tornilleria M4/M5</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Soporte antena GPS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Colin / cupula</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Mejor vista al cielo y fijacion limpia</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>ASA</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>FDM</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>+/-0.30 mm</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Resistencia UV y temperatura</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Soporte sensor velocidad</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Pinza freno / basculante</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Mantener gap estable 1.0-2.0 mm</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Nylon CF</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>SLS</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>+/-0.20 mm</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Alta rigidez para no perder calibracion</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Guia de cableado lateral</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Vigas chasis</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Ordenar mazo y evitar rozaduras</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>PETG</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>FDM</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>+/-0.30 mm</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Radio minimo en cantos para evitar rotura</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Abrazadera potenciometro</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Horquilla delantera</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Alineacion paralela y ajuste fino</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Nylon CF</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>SLS</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>+/-0.15 mm</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Validar recorrido completo de suspension</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Material / Pieza</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Especificacion Tecnica</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cantidad Est.</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Proposito de Instalacion</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Proveedor sugerido</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Referencia proveedor</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Coste estimado (EUR)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Coste total (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Soportes</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pletina de Aluminio</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Grado 6061-T6 (2mm)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1 unidad</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Soportes de Dash y Sensor Velocidad.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Soportes</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Abrazaderas de Horquilla</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Anillos mecanizados a medida</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2 unidades</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Anclaje de potenciometro a suspension.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Tornilleria</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Kit Tornilleria Inox</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Acero Inox A2 (M4, M5, M6)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Fijacion de herrajes y sensores.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Fijacion</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Velcro Industrial</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>3M Dual Lock</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>20 cm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Sujecion de EVO4 y Dash.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fijacion</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Adhesivo Doble Cara</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>3M VHB (Very High Bond)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 rollo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Fijacion de antena GPS.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cinta de Tela (Tesa)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Estilo OEM (Motorcycle)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1 rollo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion mazo de cables contra roces.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tubo Termorretractil</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Con adhesivo interno</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Sellado estanco de conexiones.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Bridas de Nylon</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Resistentes UV/Calor</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>50 unidades</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Organizacion del cableado por el chasis.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Quimicos</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Fijador de Roscas</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Loctite 243 (Azul)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1 bote</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad contra vibraciones del motor.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Quimicos</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Limpiador Superficies</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Alcohol Isopropilico</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1 bote</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Limpieza previa de zonas de contacto.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Electrico</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Porta-fusible aereo</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Mini-blade (Fusible 5A)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1 unidad</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion linea de alimentacion.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ruta relativa</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tamano (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sin STL detectados</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>